<commit_message>
trabajo_gav.xlsx: niveles actuales y nombres completos corregidos (Lluk, Besser, Vela Poo, Capitanachi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EsLdurz1dkmzTgP9Dw2L4J
</commit_message>
<xml_diff>
--- a/modulos/gav-training/trabajo_gav.xlsx
+++ b/modulos/gav-training/trabajo_gav.xlsx
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2" s="42" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="K2" s="42" t="inlineStr">
         <is>
-          <t>Joan Lluke González</t>
+          <t>Joan Lluk González</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="43" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="43" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="43" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" s="43" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C9" s="43" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" s="43" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" s="43" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="K11" s="43" t="inlineStr">
         <is>
-          <t>Santiago Camacho Becerra</t>
+          <t>Santiago Camacho Besser</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
         </is>
       </c>
       <c r="B12" s="38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="B16" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="B18" s="38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C19" s="28" t="inlineStr">
         <is>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="B21" s="38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
       <c r="B22" s="39" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="B23" s="38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
       <c r="B24" s="38" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="K24" s="29" t="inlineStr">
         <is>
-          <t>Nicolás Capitanacci Vicentín</t>
+          <t>Nicolás Capitanachi Vicentín</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
@@ -2902,10 +2902,8 @@
           <t>Alonso</t>
         </is>
       </c>
-      <c r="B27" s="24" t="inlineStr">
-        <is>
-          <t>JR FIG</t>
-        </is>
+      <c r="B27" s="24" t="n">
+        <v>10</v>
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
@@ -2974,7 +2972,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="30" t="inlineStr">
         <is>
@@ -3034,7 +3032,7 @@
       </c>
       <c r="K28" s="30" t="inlineStr">
         <is>
-          <t>Diego Emilio Vela</t>
+          <t>Diego Emilio Vela Poo</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3110,7 @@
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C30" s="30" t="inlineStr">
         <is>
@@ -3180,10 +3178,8 @@
           <t>Richie</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
-        <is>
-          <t>JR FIG</t>
-        </is>
+      <c r="B31" s="1" t="n">
+        <v>10</v>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>

</xml_diff>